<commit_message>
docs: commit all diagram updates and spec files
</commit_message>
<xml_diff>
--- a/docs/crc.xlsx
+++ b/docs/crc.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Agronomist, Operator, Storekeeper</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>FarmParticipant, Field, CropYieldAnalysis</t>
+          <t>Field, CropYieldAnalysis</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>FarmParticipant, Field, FieldWork, TechOperation, WeatherService</t>
+          <t>Field, FieldWork, TechOperation, WeatherService</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>FarmParticipant, Field</t>
+          <t>Field</t>
         </is>
       </c>
     </row>

</xml_diff>